<commit_message>
feat(dataset): ajout du premier lot de test (total 96 lignes)
</commit_message>
<xml_diff>
--- a/data/final/benchmark.xlsx
+++ b/data/final/benchmark.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S65"/>
+  <dimension ref="A1:S97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,8 +571,10 @@
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
-        <v>0</v>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -654,8 +656,10 @@
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
-        <v>0</v>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -737,8 +741,10 @@
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
-        <v>0</v>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -820,8 +826,10 @@
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
-        <v>0</v>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -903,8 +911,10 @@
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
-        <v>0</v>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -986,8 +996,10 @@
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
-        <v>0</v>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1069,8 +1081,10 @@
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
-        <v>0</v>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1152,8 +1166,10 @@
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
-        <v>0</v>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1235,8 +1251,10 @@
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
-        <v>0</v>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1318,8 +1336,10 @@
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
-        <v>0</v>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1401,8 +1421,10 @@
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
-        <v>0</v>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1484,8 +1506,10 @@
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
-        <v>0</v>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1567,8 +1591,10 @@
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
-        <v>0</v>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1650,8 +1676,10 @@
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
-        <v>0</v>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1733,8 +1761,10 @@
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>0</v>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1816,8 +1846,10 @@
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
-        <v>0</v>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1899,8 +1931,10 @@
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
-        <v>0</v>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1982,8 +2016,10 @@
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
-        <v>0</v>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2065,8 +2101,10 @@
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
-        <v>0</v>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2148,8 +2186,10 @@
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
-        <v>0</v>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2215,8 +2255,10 @@
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="n">
-        <v>0</v>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -2282,8 +2324,10 @@
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="n">
-        <v>0</v>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2349,8 +2393,10 @@
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
-        <v>0</v>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2416,8 +2462,10 @@
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="n">
-        <v>0</v>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -2483,8 +2531,10 @@
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
-        <v>0</v>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2550,8 +2600,10 @@
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="n">
-        <v>0</v>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2617,8 +2669,10 @@
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="n">
-        <v>0</v>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2684,8 +2738,10 @@
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="n">
-        <v>0</v>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2751,8 +2807,10 @@
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
-        <v>0</v>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2818,8 +2876,10 @@
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="n">
-        <v>0</v>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -2885,8 +2945,10 @@
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="n">
-        <v>0</v>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -2952,8 +3014,10 @@
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="n">
-        <v>0</v>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3019,8 +3083,10 @@
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="n">
-        <v>0</v>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3086,8 +3152,10 @@
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="n">
-        <v>0</v>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -3153,8 +3221,10 @@
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="n">
-        <v>0</v>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3220,8 +3290,10 @@
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="n">
-        <v>0</v>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -3287,8 +3359,10 @@
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="n">
-        <v>0</v>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -3354,8 +3428,10 @@
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="n">
-        <v>0</v>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -3421,8 +3497,10 @@
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="n">
-        <v>0</v>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -3488,8 +3566,10 @@
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="n">
-        <v>0</v>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -3555,8 +3635,10 @@
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="n">
-        <v>0</v>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -3622,8 +3704,10 @@
         </is>
       </c>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="n">
-        <v>0</v>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -3689,8 +3773,10 @@
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="n">
-        <v>0</v>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -3756,8 +3842,10 @@
         </is>
       </c>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="n">
-        <v>0</v>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3823,8 +3911,10 @@
           <t>3jbni had lfilm bzzaf.|3jebni had l film bzaf.</t>
         </is>
       </c>
-      <c r="N46" t="n">
-        <v>0</v>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3886,8 +3976,10 @@
         </is>
       </c>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="n">
-        <v>0</v>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -3953,8 +4045,10 @@
           <t>fin ghati tmchi fhad l3otla?|fen ghadi tmchi f had l3otla?</t>
         </is>
       </c>
-      <c r="N48" t="n">
-        <v>0</v>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -4016,8 +4110,10 @@
         </is>
       </c>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" t="n">
-        <v>0</v>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -4083,8 +4179,10 @@
           <t>lmakla dial had resto bnina w nqiya.</t>
         </is>
       </c>
-      <c r="N50" t="n">
-        <v>0</v>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -4146,8 +4244,10 @@
         </is>
       </c>
       <c r="M51" t="inlineStr"/>
-      <c r="N51" t="n">
-        <v>0</v>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -4213,8 +4313,10 @@
           <t>makrehtch nchrob kas d atay mche7er.</t>
         </is>
       </c>
-      <c r="N52" t="n">
-        <v>0</v>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -4276,8 +4378,10 @@
         </is>
       </c>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="n">
-        <v>0</v>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -4343,8 +4447,10 @@
           <t>sme7liya, wach kat3ref fin kayn lbank?</t>
         </is>
       </c>
-      <c r="N54" t="n">
-        <v>0</v>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -4406,8 +4512,10 @@
         </is>
       </c>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" t="n">
-        <v>0</v>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -4473,8 +4581,10 @@
           <t>bghit nmchi l sou9 bekri.|bghit nmchi lsou9 bkri.</t>
         </is>
       </c>
-      <c r="N56" t="n">
-        <v>0</v>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -4536,8 +4646,10 @@
         </is>
       </c>
       <c r="M57" t="inlineStr"/>
-      <c r="N57" t="n">
-        <v>0</v>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -4603,8 +4715,10 @@
           <t>chhal kaydir had lkilo dial teffah?|ch7al kidir had lkilo d tfa7?</t>
         </is>
       </c>
-      <c r="N58" t="n">
-        <v>0</v>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -4666,8 +4780,10 @@
         </is>
       </c>
       <c r="M59" t="inlineStr"/>
-      <c r="N59" t="n">
-        <v>0</v>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -4733,8 +4849,10 @@
           <t>bghit nsowlk 3la lwa9t dl khedma ghdda.|bghit nsewlek 3la taw9it dial lkhdma ghda.</t>
         </is>
       </c>
-      <c r="N60" t="n">
-        <v>0</v>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -4796,8 +4914,10 @@
         </is>
       </c>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" t="n">
-        <v>0</v>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
@@ -4863,8 +4983,10 @@
           <t>tbarkellah 3lik, rak khdemti mezyan f had lmachro3.</t>
         </is>
       </c>
-      <c r="N62" t="n">
-        <v>0</v>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -4926,8 +5048,10 @@
         </is>
       </c>
       <c r="M63" t="inlineStr"/>
-      <c r="N63" t="n">
-        <v>0</v>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -4993,8 +5117,10 @@
           <t>kantmna lik tawfiq w najah f limti7an dialk.|kantmenna lik tawfi9 w naja7.</t>
         </is>
       </c>
-      <c r="N64" t="n">
-        <v>0</v>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -5056,30 +5182,2352 @@
         </is>
       </c>
       <c r="M65" t="inlineStr"/>
-      <c r="N65" t="n">
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Q-011</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>حميد ضرّاتو ضرسة العقل، مشا عند دونتيست فالعشية حيدها ليه وعطاه الدوا.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>شنو دار حميد عند الطبيب؟</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>دار راديو لرجلو</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>عبر الطانسيو</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>حيد ضرسة العقل</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>دار عملية على عينو</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="n">
         <v>0</v>
       </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>original</t>
-        </is>
-      </c>
-      <c r="P65" t="inlineStr">
-        <is>
-          <t>éducation</t>
-        </is>
-      </c>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>easy</t>
-        </is>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="S65" t="inlineStr"/>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Q-011</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>7mid derrato dersat l39el, mcha 3nd dentiste f l3chiya 7yedha lih w 3tah ddwa.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Chnou dar 7mid 3nd tbib?</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>dar radio l rejlou</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>3ber ttansyou</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>7yed dersat l39el</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>dar 3amaliya 3la 3aynou</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Q-012</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>رشيد مشا للمقاطعة باش يصادق على العقد، لقا الزحام بزاف وتسنى نوبتو حتى لتماش.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>علاش مشا رشيد للمقاطعة؟</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>باش يليزالي العقد</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>باش يجدد الباسبور</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>باش يشري طوموبيل</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>باش يدفع للفيزا</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Q-012</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Rachid mcha l lmo9ata3a bach yssade9 3la l3a9d, l9a zze7am bzaf w tsenna noubto 7tta ltmmach.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>3lach mcha Rachid l lmo9ata3a?</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>bach ylegaliser l3a9d</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>bach yjedded lbasspor</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>bach ychri tomobil</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>bach ydfa3 l visa</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Q-013</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>المنتخب المغربي ربح الماتش بجوج لواحد، وسجل النصيري هدف واعر بالراس فالشوط الثاني.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>كيفاش تسجل الهدف ديال النصيري؟</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ببيلانتي</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>بتير من بعيد</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>ضد مرماه</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>بالراس</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Q-013</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Lmontakhab lmoghribi rbe7 lmatch b jouj l wa7ed, w sejjel En-Nesyri hadaf wa3er b rras f chawt ttani.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Kifach tsejjel lhadaf dyal En-Nesyri?</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>b penalty</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>b tir mn b3id</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>dedd marmatou</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>b rras</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Q-014</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>نهار الجمعة، جمعات الوالدة العائلة كلها ودارت ليهم قصعة د كسكسو بالسبع خضاري واللبن.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>شنو وجدات الوالدة نهار الجمعة؟</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>طاجين د الحوت</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>قصعة د كسكسو باللبن</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>بسطيلة د الدجاج</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>رفيسة بالحلية</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Q-014</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Nhar jjomo3a, jem3at lwalida l3a2ila kamla w daret lihom 9es3a d ksekso b sbe3 khdari w lben.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Chnou wejdat lwalida nhar jjomo3a?</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>tajin d l7out</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>9es3a d ksekso b lben</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>pastilla d ddjaj</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>rfissa b l7elba</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Q-015</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>طاحت الشتا خيط من السما، الشوارع فايضين والناس هازين المظلات كيجريو للديور.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>كيفاش كان الحال على برا؟</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>الشتا خيط من السما</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>الصهد والشمس حارة</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>الثلج كيطيح بزاف</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>العجاج والغبرة</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>météo</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Q-015</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Ta7et chta khit mn ssma, chawari3 faydin w nass hazin lmdallat kayjriw l ddyour.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Kifach kan l7al 3la berra?</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>chta khit mn ssma</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>sshed w chems 7arra</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>ttelj kayti7 bzaf</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>l3jaj w lghobra</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>météo</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Q-016</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>التلفون ديال أنس طاح ليه فالما وتطفى، داه للمصلح بدّل ليه لافيشور ورجع خدام.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>شنو بدّل المصلح فالتلفون؟</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>الباتري</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>الباف د الصوت</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>لافيشور</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>الكاميرا</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>technologie</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Q-016</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Ttilifoun dyal Anass ta7 lih f lma w ttfa, ddah l lmosli7 beddel lih l'afficheur w rje3 khddam.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Chnou beddel lmosli7 f ttilifoun?</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>lbattrie</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>lbaf d ssawt</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>l'afficheur</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>lkamera</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>technologie</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>N-005a</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>أمين جاب الباك بميزة حسن جدا وفرحات العائلة.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>أمين نجح فالامتحان د الباك.</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>N-005a</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Amine jab lbac b mizat 7assan jiddan w fer7at l3a2ila.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Amine nje7 f lmtihan d lbac.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>N-005b</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>أمين جاب الباك بميزة حسن جدا وفرحات العائلة.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>أمين سقط فهاد العام.</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>N-005b</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Amine jab lbac b mizat 7assan jiddan w fer7at l3a2ila.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Amine s9et f had l3am.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>N-005c</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>أمين جاب الباك بميزة حسن جدا وفرحات العائلة.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>أمين غادي يدير كلية الطب العام الجاي.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>N-005c</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Amine jab lbac b mizat 7assan jiddan w fer7at l3a2ila.</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Amine ghadi ydir kolliyat ttibb l3am jjay.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>N-006a</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>سلمى ركبات فالطيارة متوجهة لتركيا باش تدوز العطلة.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>سلمى مسافرة خارج المغرب.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>N-006a</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Salma rekbat f ttiyara motawajjiha l Tourkia bach ddozewez l3otla.</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Salma msafra kharij lmoghrib.</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>N-006b</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>سلمى ركبات فالطيارة متوجهة لتركيا باش تدوز العطلة.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>سلمى باقا كالسة فدارهم فكازا.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>N-006b</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Salma rekbat f ttiyara motawajjiha l Tourkia bach ddozewez l3otla.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Salma ba9a galsa f darhom f Casa.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>N-006c</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>سلمى ركبات فالطيارة متوجهة لتركيا باش تدوز العطلة.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>سلمى كتعرف تهضر بالتركية مزيان.</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="n">
+        <v>0</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>N-006c</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Salma rekbat f ttiyara motawajjiha l Tourkia bach ddozewez l3otla.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Salma kat3ref thder b ttourkia mzyan.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>voyage</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>C-011</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>فين وصلتي، راني كنتسناك حدا المحطة.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Fin wselti, rani kantsnak 7da lma7atta.</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>fin wsliti, rani kantsenak 7da lmahata.|fen wselti rani kantsnak.</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>vie courante</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>C-011</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Fin wselti, rani kantsnak 7da lma7atta.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>فين وصلتي، راني كنتسناك حدا المحطة.</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>vie courante</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>C-012</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>خاصك تشرب الدوا فوقتو وتبع الريجيم.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Khassek tchreb ddwa f we9to w ttebbe3 rrijim.</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>khasek tchrob dwa f weqto w tebe3 rijim.|khask tchreb ddwa.</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>C-012</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Khassek tchreb ddwa f we9to w ttebbe3 rrijim.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>خاصك تشرب الدوا فوقتو وتبع الريجيم.</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>C-013</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>صيفط ليا الإيميل باش نشوف الدوسي اليوم.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Seyfet lia l'email bach nchouf ddossier lyoma.</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>sift liya l email bach nchof dossier lyom.|sayfet lia l'email.</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>C-013</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Seyfet lia l'email bach nchouf ddossier lyoma.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>صيفط ليا الإيميل باش نشوف الدوسي اليوم.</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="n">
+        <v>0</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>C-014</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>عفاك شحال الحساب كامل؟</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>3afak ch7al l7ssab kamel?</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>3afak chhal lhesab kamel?|3afak ch7al le7ssab kamel?</t>
+        </is>
+      </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>achats</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>C-014</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>3afak ch7al l7ssab kamel?</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>عفاك شحال الحساب كامل؟</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="n">
+        <v>0</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>achats</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(dataset): ajout lot 2 de test - benchmark à 124 lignes validé
</commit_message>
<xml_diff>
--- a/data/final/benchmark.xlsx
+++ b/data/final/benchmark.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S97"/>
+  <dimension ref="A1:S125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5267,8 +5267,10 @@
         </is>
       </c>
       <c r="M66" t="inlineStr"/>
-      <c r="N66" t="n">
-        <v>0</v>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -5350,8 +5352,10 @@
         </is>
       </c>
       <c r="M67" t="inlineStr"/>
-      <c r="N67" t="n">
-        <v>0</v>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -5433,8 +5437,10 @@
         </is>
       </c>
       <c r="M68" t="inlineStr"/>
-      <c r="N68" t="n">
-        <v>0</v>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -5516,8 +5522,10 @@
         </is>
       </c>
       <c r="M69" t="inlineStr"/>
-      <c r="N69" t="n">
-        <v>0</v>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -5599,8 +5607,10 @@
         </is>
       </c>
       <c r="M70" t="inlineStr"/>
-      <c r="N70" t="n">
-        <v>0</v>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -5682,8 +5692,10 @@
         </is>
       </c>
       <c r="M71" t="inlineStr"/>
-      <c r="N71" t="n">
-        <v>0</v>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -5765,8 +5777,10 @@
         </is>
       </c>
       <c r="M72" t="inlineStr"/>
-      <c r="N72" t="n">
-        <v>0</v>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -5848,8 +5862,10 @@
         </is>
       </c>
       <c r="M73" t="inlineStr"/>
-      <c r="N73" t="n">
-        <v>0</v>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -5931,8 +5947,10 @@
         </is>
       </c>
       <c r="M74" t="inlineStr"/>
-      <c r="N74" t="n">
-        <v>0</v>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
@@ -6014,8 +6032,10 @@
         </is>
       </c>
       <c r="M75" t="inlineStr"/>
-      <c r="N75" t="n">
-        <v>0</v>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O75" t="inlineStr">
         <is>
@@ -6097,8 +6117,10 @@
         </is>
       </c>
       <c r="M76" t="inlineStr"/>
-      <c r="N76" t="n">
-        <v>0</v>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -6180,8 +6202,10 @@
         </is>
       </c>
       <c r="M77" t="inlineStr"/>
-      <c r="N77" t="n">
-        <v>0</v>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -6247,8 +6271,10 @@
         </is>
       </c>
       <c r="M78" t="inlineStr"/>
-      <c r="N78" t="n">
-        <v>0</v>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -6314,8 +6340,10 @@
         </is>
       </c>
       <c r="M79" t="inlineStr"/>
-      <c r="N79" t="n">
-        <v>0</v>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -6381,8 +6409,10 @@
         </is>
       </c>
       <c r="M80" t="inlineStr"/>
-      <c r="N80" t="n">
-        <v>0</v>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -6448,8 +6478,10 @@
         </is>
       </c>
       <c r="M81" t="inlineStr"/>
-      <c r="N81" t="n">
-        <v>0</v>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O81" t="inlineStr">
         <is>
@@ -6515,8 +6547,10 @@
         </is>
       </c>
       <c r="M82" t="inlineStr"/>
-      <c r="N82" t="n">
-        <v>0</v>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O82" t="inlineStr">
         <is>
@@ -6582,8 +6616,10 @@
         </is>
       </c>
       <c r="M83" t="inlineStr"/>
-      <c r="N83" t="n">
-        <v>0</v>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -6649,8 +6685,10 @@
         </is>
       </c>
       <c r="M84" t="inlineStr"/>
-      <c r="N84" t="n">
-        <v>0</v>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O84" t="inlineStr">
         <is>
@@ -6716,8 +6754,10 @@
         </is>
       </c>
       <c r="M85" t="inlineStr"/>
-      <c r="N85" t="n">
-        <v>0</v>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O85" t="inlineStr">
         <is>
@@ -6783,8 +6823,10 @@
         </is>
       </c>
       <c r="M86" t="inlineStr"/>
-      <c r="N86" t="n">
-        <v>0</v>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -6850,8 +6892,10 @@
         </is>
       </c>
       <c r="M87" t="inlineStr"/>
-      <c r="N87" t="n">
-        <v>0</v>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -6917,8 +6961,10 @@
         </is>
       </c>
       <c r="M88" t="inlineStr"/>
-      <c r="N88" t="n">
-        <v>0</v>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -6984,8 +7030,10 @@
         </is>
       </c>
       <c r="M89" t="inlineStr"/>
-      <c r="N89" t="n">
-        <v>0</v>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -7051,8 +7099,10 @@
           <t>fin wsliti, rani kantsenak 7da lmahata.|fen wselti rani kantsnak.</t>
         </is>
       </c>
-      <c r="N90" t="n">
-        <v>0</v>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -7114,8 +7164,10 @@
         </is>
       </c>
       <c r="M91" t="inlineStr"/>
-      <c r="N91" t="n">
-        <v>0</v>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -7181,8 +7233,10 @@
           <t>khasek tchrob dwa f weqto w tebe3 rijim.|khask tchreb ddwa.</t>
         </is>
       </c>
-      <c r="N92" t="n">
-        <v>0</v>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -7244,8 +7298,10 @@
         </is>
       </c>
       <c r="M93" t="inlineStr"/>
-      <c r="N93" t="n">
-        <v>0</v>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -7311,8 +7367,10 @@
           <t>sift liya l email bach nchof dossier lyom.|sayfet lia l'email.</t>
         </is>
       </c>
-      <c r="N94" t="n">
-        <v>0</v>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O94" t="inlineStr">
         <is>
@@ -7374,8 +7432,10 @@
         </is>
       </c>
       <c r="M95" t="inlineStr"/>
-      <c r="N95" t="n">
-        <v>0</v>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O95" t="inlineStr">
         <is>
@@ -7441,8 +7501,10 @@
           <t>3afak chhal lhesab kamel?|3afak ch7al le7ssab kamel?</t>
         </is>
       </c>
-      <c r="N96" t="n">
-        <v>0</v>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -7504,30 +7566,2020 @@
         </is>
       </c>
       <c r="M97" t="inlineStr"/>
-      <c r="N97" t="n">
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>achats</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Q-017</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>طارق مشا لكيشي أوطوماتيك باش يخرج الفلوس، لقا الكارت تبلوكات حيت غلط فالمودباس تلاتة د المرات.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>علاش تبلوكات لاكارت د طارق؟</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>حيت الماكينة خاسرة</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>حيت سالاو الفلوس</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>حيت غلط فالمودباس تلاتة د المرات</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>حيت ضاعت ليه لاكارت</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="n">
         <v>0</v>
       </c>
-      <c r="O97" t="inlineStr">
-        <is>
-          <t>original</t>
-        </is>
-      </c>
-      <c r="P97" t="inlineStr">
-        <is>
-          <t>achats</t>
-        </is>
-      </c>
-      <c r="Q97" t="inlineStr">
-        <is>
-          <t>easy</t>
-        </is>
-      </c>
-      <c r="R97" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="S97" t="inlineStr"/>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>banque</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Q-017</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Tariq mcha l guichet automatique bach ykherrej lflous, l9a la carte tbloukat 7it ghlet f mot de passe tlata d lmarrat.</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>3lach tbloukat la carte d Tariq?</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>7it lmakina khasra</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>7it salaw lflous</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>7it ghlet f mot de passe tlata d lmarrat</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>7it da3et lih la carte</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="n">
+        <v>0</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>banque</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Q-018</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>سعاد شرات زربية تقليدية د تازناخت من المدينة القديمة ف فاس، صاوبوها بالصوف الحر والألوان الطبيعية.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>باش تصاوبات الزربية لي شرات سعاد؟</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>بالحرير والبلاستيك</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>بالقطن والخيط العادي</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>بالجلد والكتان</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>بالصوف الحر والألوان الطبيعية</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="n">
+        <v>0</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>artisanat</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Q-018</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Souad chrat zerbiya ta9lidiya d Taznakht mn lmdina l9dima f Fes, sawbouha b ssouf l7orr w l'alwan ttabi3iya.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Bach tsawbat zzerbiya li chrat Souad?</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>b l7rir w lplastique</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>b l9ten w lkhit l3adi</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>b ljelda w lkettan</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>b ssouf l7orr w l'alwan ttabi3iya</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="n">
+        <v>0</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>artisanat</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Q-019</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>الطلبة كراو برطمة قريبة للفاك ب تلتالاف درهم للشهر، مقسومة عليهم بربعة ومفرشة كاملة.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>بشحال كراو الطلبة البرطمة؟</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>ب تلتالاف درهم للشهر</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>ب ألف درهم للشهر</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>ب خمسالاف درهم للشهر</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>فابور بلا خلاص</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="n">
+        <v>0</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>logement</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Q-019</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Ttolaba kraw bpartma 9riba l la fac b teltalaf derham l chher, ma9souma 3lihom b rebya w mferrcha kamla.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Bch7al kraw ttolaba lpartma?</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>b teltalaf derham l chher</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>b alf derham l chher</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>b khmstalaf derham l chher</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>fabor bla khlas</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="n">
+        <v>0</v>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>logement</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Q-020</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>ملي كان هشام صايغ فلوطوروت، تفشات ليه الرويضة الورانية، وقف فالبان ديرجونس وبدلها بالسوكوندير.</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>شنو وقع لطوموبيل د هشام؟</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>سالات ليها ليسانس</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>تفشات الرويضة الورانية</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>تكسرات الزاجة القدامية</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>سخن ليها الموطور</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>automobile</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Q-020</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Mlli kan Hicham saye9 f l'autoroute, tefchat lih rrwida lworaniya, w9ef f la bande d'urgence w beddelha b ssekondair.</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Chnou w9e3 l tomobil d Hicham?</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>salat liha l'essence</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>tefchat rrwida lworaniya</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>tkessrat zzaja l9ddamiya</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>skhen liha lmoteur</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="n">
+        <v>0</v>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>automobile</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>N-007a</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>المهدي كيمشي لاصال كل نهار كيهز الثقال وكيجري نص ساعة.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>المهدي كيمارس الرياضة.</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="n">
+        <v>0</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>N-007a</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Lmehdi kaymchi l la salle kol nhar kayhez tte9al w kayjri noss sa3a.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Lmehdi kaymares rriyada.</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="n">
+        <v>0</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>N-007b</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>المهدي كيمشي لاصال كل نهار كيهز الثقال وكيجري نص ساعة.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>المهدي جالس فالدار ما كيتحركش.</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>N-007b</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Lmehdi kaymchi l la salle kol nhar kayhez tte9al w kayjri noss sa3a.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Lmehdi jales f ddar ma kayt7errekch.</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>N-007c</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>المهدي كيمشي لاصال كل نهار كيهز الثقال وكيجري نص ساعة.</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>المهدي متبع ريجيم فيه البروتين بزاف.</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>N-007c</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Lmehdi kaymchi l la salle kol nhar kayhez tte9al w kayjri noss sa3a.</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Lmehdi mtbe3 rijim fih lprotein bzaf.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="n">
+        <v>0</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>N-008a</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>خديجة دفعت تكشيطة عند الخياط باش توجدها لعرس ختها السيمانة الجاية.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>أخت خديجة غادا تزوج قريبا.</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="n">
+        <v>0</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>fêtes</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>N-008a</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Khadija def3at tekchita 3nd lkheyat bach twjedha l 3ers kht-ha simana jjaya.</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Kht Khadija ghada tzwwej 9riban.</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="n">
+        <v>0</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>fêtes</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>N-008b</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>خديجة دفعت تكشيطة عند الخياط باش توجدها لعرس ختها السيمانة الجاية.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>خديجة ما عندها حتى مناسبة عائلية.</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="n">
+        <v>0</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>fêtes</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>N-008b</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Khadija def3at tekchita 3nd lkheyat bach twjedha l 3ers kht-ha simana jjaya.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Khadija ma 3ndha 7tta mounasaba 3a2iliya.</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="n">
+        <v>0</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>fêtes</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>N-008c</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>خديجة دفعت تكشيطة عند الخياط باش توجدها لعرس ختها السيمانة الجاية.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>التكشيطة لونها خضر ملكي ومطروزة بالصقلي.</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="n">
+        <v>0</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>fêtes</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>N-008c</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Khadija def3at tekchita 3nd lkheyat bach twjedha l 3ers kht-ha simana jjaya.</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Ttekchita lwnha khder malaki w mtrouza b sse9li.</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="n">
+        <v>0</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>fêtes</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>C-015</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>الله يعطيك الصحة على هاد المجهود.</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Llah ya3tik sse77a 3la had lmajhoub.</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>llah y3tik saha 3la had lmejhoud.|lah ya3tik se7a.</t>
+        </is>
+      </c>
+      <c r="N118" t="n">
+        <v>0</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>quotidien</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>C-015</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Llah ya3tik sse77a 3la had lmajhoub.</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>الله يعطيك الصحة على هاد المجهود.</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>quotidien</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>C-016</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>كاين واحد الصهد صعيب اليوم فالزنقة.</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Kayen wa7ed sshed s3ib lyoma f zzen9a.</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>kayn wahd shed s3ib lyom f zanqa.|kayn wahed sehd s3ib.</t>
+        </is>
+      </c>
+      <c r="N120" t="n">
+        <v>0</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>météo</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>C-016</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Kayen wa7ed sshed s3ib lyoma f zzen9a.</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>كاين واحد الصهد صعيب اليوم فالزنقة.</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>météo</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>C-017</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>سلم ليا على الوالد والدار كاملين.</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Sellem lia 3la lwalid w ddar kamlin.</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>slem liya 3la lwalid w dar kamlin.|sellem 3la lwalid.</t>
+        </is>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>famille</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>C-017</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Sellem lia 3la lwalid w ddar kamlin.</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>سلم ليا على الوالد والدار كاملين.</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="n">
+        <v>0</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>famille</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>C-018</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>واش عندك الصرف ديال ميتين درهم؟</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Wach 3ndek ssarf dyal miyatayn derham?</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>wach 3ndk sarf dial 200 derham?|wach 3ndek ssarf d mitin drhm?</t>
+        </is>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>commerce</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>C-018</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Wach 3ndek ssarf dyal miyatayn derham?</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>واش عندك الصرف ديال ميتين درهم؟</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>commerce</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(dataset): benchmark complet validé (156 lignes - Dev & Test)
</commit_message>
<xml_diff>
--- a/data/final/benchmark.xlsx
+++ b/data/final/benchmark.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S125"/>
+  <dimension ref="A1:S157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7651,8 +7651,10 @@
         </is>
       </c>
       <c r="M98" t="inlineStr"/>
-      <c r="N98" t="n">
-        <v>0</v>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -7734,8 +7736,10 @@
         </is>
       </c>
       <c r="M99" t="inlineStr"/>
-      <c r="N99" t="n">
-        <v>0</v>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -7817,8 +7821,10 @@
         </is>
       </c>
       <c r="M100" t="inlineStr"/>
-      <c r="N100" t="n">
-        <v>0</v>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -7900,8 +7906,10 @@
         </is>
       </c>
       <c r="M101" t="inlineStr"/>
-      <c r="N101" t="n">
-        <v>0</v>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -7983,8 +7991,10 @@
         </is>
       </c>
       <c r="M102" t="inlineStr"/>
-      <c r="N102" t="n">
-        <v>0</v>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -8066,8 +8076,10 @@
         </is>
       </c>
       <c r="M103" t="inlineStr"/>
-      <c r="N103" t="n">
-        <v>0</v>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -8149,8 +8161,10 @@
         </is>
       </c>
       <c r="M104" t="inlineStr"/>
-      <c r="N104" t="n">
-        <v>0</v>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -8232,8 +8246,10 @@
         </is>
       </c>
       <c r="M105" t="inlineStr"/>
-      <c r="N105" t="n">
-        <v>0</v>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -8299,8 +8315,10 @@
         </is>
       </c>
       <c r="M106" t="inlineStr"/>
-      <c r="N106" t="n">
-        <v>0</v>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -8366,8 +8384,10 @@
         </is>
       </c>
       <c r="M107" t="inlineStr"/>
-      <c r="N107" t="n">
-        <v>0</v>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O107" t="inlineStr">
         <is>
@@ -8433,8 +8453,10 @@
         </is>
       </c>
       <c r="M108" t="inlineStr"/>
-      <c r="N108" t="n">
-        <v>0</v>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -8500,8 +8522,10 @@
         </is>
       </c>
       <c r="M109" t="inlineStr"/>
-      <c r="N109" t="n">
-        <v>0</v>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -8567,8 +8591,10 @@
         </is>
       </c>
       <c r="M110" t="inlineStr"/>
-      <c r="N110" t="n">
-        <v>0</v>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -8634,8 +8660,10 @@
         </is>
       </c>
       <c r="M111" t="inlineStr"/>
-      <c r="N111" t="n">
-        <v>0</v>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -8701,8 +8729,10 @@
         </is>
       </c>
       <c r="M112" t="inlineStr"/>
-      <c r="N112" t="n">
-        <v>0</v>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -8768,8 +8798,10 @@
         </is>
       </c>
       <c r="M113" t="inlineStr"/>
-      <c r="N113" t="n">
-        <v>0</v>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -8835,8 +8867,10 @@
         </is>
       </c>
       <c r="M114" t="inlineStr"/>
-      <c r="N114" t="n">
-        <v>0</v>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -8902,8 +8936,10 @@
         </is>
       </c>
       <c r="M115" t="inlineStr"/>
-      <c r="N115" t="n">
-        <v>0</v>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -8969,8 +9005,10 @@
         </is>
       </c>
       <c r="M116" t="inlineStr"/>
-      <c r="N116" t="n">
-        <v>0</v>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -9036,8 +9074,10 @@
         </is>
       </c>
       <c r="M117" t="inlineStr"/>
-      <c r="N117" t="n">
-        <v>0</v>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -9103,8 +9143,10 @@
           <t>llah y3tik saha 3la had lmejhoud.|lah ya3tik se7a.</t>
         </is>
       </c>
-      <c r="N118" t="n">
-        <v>0</v>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O118" t="inlineStr">
         <is>
@@ -9166,8 +9208,10 @@
         </is>
       </c>
       <c r="M119" t="inlineStr"/>
-      <c r="N119" t="n">
-        <v>0</v>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -9233,8 +9277,10 @@
           <t>kayn wahd shed s3ib lyom f zanqa.|kayn wahed sehd s3ib.</t>
         </is>
       </c>
-      <c r="N120" t="n">
-        <v>0</v>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O120" t="inlineStr">
         <is>
@@ -9296,8 +9342,10 @@
         </is>
       </c>
       <c r="M121" t="inlineStr"/>
-      <c r="N121" t="n">
-        <v>0</v>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -9363,8 +9411,10 @@
           <t>slem liya 3la lwalid w dar kamlin.|sellem 3la lwalid.</t>
         </is>
       </c>
-      <c r="N122" t="n">
-        <v>0</v>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -9426,8 +9476,10 @@
         </is>
       </c>
       <c r="M123" t="inlineStr"/>
-      <c r="N123" t="n">
-        <v>0</v>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O123" t="inlineStr">
         <is>
@@ -9493,8 +9545,10 @@
           <t>wach 3ndk sarf dial 200 derham?|wach 3ndek ssarf d mitin drhm?</t>
         </is>
       </c>
-      <c r="N124" t="n">
-        <v>0</v>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O124" t="inlineStr">
         <is>
@@ -9556,30 +9610,2280 @@
         </is>
       </c>
       <c r="M125" t="inlineStr"/>
-      <c r="N125" t="n">
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>commerce</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Q-021</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>سلوى مشات لسنتر فيل تشري كادو لعيد ميلاد ختها، لقات صاك جلد كحل واعر وشراتو.</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>شنو شرات سلوى كادو لختها؟</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>خاتم د الذهب</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>ساعة يد</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>ريحة غالية</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>صاك جلد كحل</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="n">
         <v>0</v>
       </c>
-      <c r="O125" t="inlineStr">
-        <is>
-          <t>original</t>
-        </is>
-      </c>
-      <c r="P125" t="inlineStr">
-        <is>
-          <t>commerce</t>
-        </is>
-      </c>
-      <c r="Q125" t="inlineStr">
-        <is>
-          <t>easy</t>
-        </is>
-      </c>
-      <c r="R125" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="S125" t="inlineStr"/>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>achats</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Q-021</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Salwa mchat l centre-ville tchri cadeau l 3id milad kht-ha, l9at sac jeld k7el wa3er w chratou.</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Chnou chrat Salwa cadeau l kht-ha?</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>khatem d ddheb</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>sa3a d lyed</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>ri7a ghalya</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>sac jeld k7el</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>achats</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Q-022</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>الطاكسي كبير وقف فالرونبوان باش يركب الناس، وبقات بلاصة وحدة اللور خاوية.</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>فين بقات البلاصة الخاوية فالطاكسي؟</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>بقات بلاصة وحدة اللور</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>القدام حدا الشيفور</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>فالملا فالسقف</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>الطاكسي كان عامر كلو</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="n">
+        <v>0</v>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Q-022</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Ttaxi kbir w9ef f rond-point bach yrkkeb nass, w b9at blassa we7da llour khawya.</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Fin b9at lblassa lkhawya f ttaxi?</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>b9at blassa we7da llour</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>l9ddam 7da chifour</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>f lmalla f sse9f</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ttaxi kan 3amer kollou</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr"/>
+      <c r="N129" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Q-023</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>مشاو الدراري للبحر فالصيف، لقاوه عامر والموج عالي بزاف حيت كان الريح الشرقي.</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>علاش كان الموج عالي فالبحر؟</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>حيت الما كان بارد</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>حيت طاحت الشتا</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>حيت كان الريح الشرقي</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>حيت الليل قرب يطيح</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr"/>
+      <c r="N130" t="n">
+        <v>0</v>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>météo</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Q-023</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Mchaw ddrari l lb7ar f ssif, l9awh 3amer w lmouj 3ali bzaf 7it kan rri7 cher9i.</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>3lach kan lmouj 3ali f lb7ar?</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>7it lma kan bared</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>7it ta7et chta</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>7it kan rri7 cher9i</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>7it llil 9reb yti7</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr"/>
+      <c r="N131" t="n">
+        <v>0</v>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>météo</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Q-024</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>جواد نسى السوارت فوق الطابلة فالكوزينة، وملي خرج وسد الباب عاد تفكرهم وبقا واحل.</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>فين نسى جواد السوارت؟</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>فالطوموبيل</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>فالجيب د الجاكيتة</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>فالخدمة</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>فوق الطابلة فالكوزينة</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr"/>
+      <c r="N132" t="n">
+        <v>0</v>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>vie quotidienne</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Q-024</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Jawad nsa sswaret fo9 ttabla f lkouzina, w mlli khrej w sedd lbab 3ad tfekkerhom w b9a wa7el.</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Fin nsa Jawad sswaret?</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>f tomobil</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>f jjib d ljakita</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>f lkhedma</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>fo9 ttabla f lkouzina</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr"/>
+      <c r="N133" t="n">
+        <v>0</v>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>vie quotidienne</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>N-011a</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>إيمان كطيب طاجين ديال الحوت فالفران.</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>إيمان كتوجد الماكلة.</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr"/>
+      <c r="N134" t="n">
+        <v>0</v>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>N-011a</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Imane katyeb tajin dyal l7out f lferran.</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Imane katwjed lmakla.</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="n">
+        <v>0</v>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>N-011b</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>إيمان كطيب طاجين ديال الحوت فالفران.</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>إيمان معمرها دخلات للكوزينة.</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr"/>
+      <c r="N136" t="n">
+        <v>0</v>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>N-011b</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Imane katyeb tajin dyal l7out f lferran.</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Imane m3mmrha dekhlat l lkouzina.</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>N-011c</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>إيمان كطيب طاجين ديال الحوت فالفران.</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>الحوت لي دارت هو الصول.</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr"/>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>N-011c</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Imane katyeb tajin dyal l7out f lferran.</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>L7out li daret houwa sole.</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>N-012a</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>بلال جاب النقطة اللولة فالمات فالقسم كامل.</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>بلال كيقرا مزيان الماط.</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>N-012a</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Bilal jab nno9ta loullya f lmath f l9ism kamel.</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Bilal kay9ra mzyan lmath.</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>N-012b</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>بلال جاب النقطة اللولة فالمات فالقسم كامل.</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>بلال هو اللخر فالماط فالقسم.</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>N-012b</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Bilal jab nno9ta loullya f lmath f l9ism kamel.</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Bilal houwa llekher f lmath f l9ism.</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr"/>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>N-012c</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>بلال جاب النقطة اللولة فالمات فالقسم كامل.</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>بلال باغي يدير مهندس د لانفورماتيك.</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr"/>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>N-012c</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Bilal jab nno9ta loullya f lmath f l9ism kamel.</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Bilal baghi ydir ingénieur d l'informatique.</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="n">
+        <v>0</v>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>C-019</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>ما بقاش فيا الحال، المهم هي الصحة والسلامة.</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Ma b9ach fiya l7al, lmouhim hiya sse77a w ssalama.</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>mab9ach fia lhal, lmohim hya seha w salama.|ma b9ach fiya lhal.</t>
+        </is>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>C-019</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Ma b9ach fiya l7al, lmouhim hiya sse77a w ssalama.</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>ما بقاش فيا الحال، المهم هي الصحة والسلامة.</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="n">
+        <v>0</v>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>C-020</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>واش هاد الطوبيس كيدوز على جامع الفنا؟</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Wach had ttobis kaydouz 3la Jame3 lfna?</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>wach had tobis kidouz 3la jama3 lfna?|wach had ttobis kaydoz 3la jame3 lfna?</t>
+        </is>
+      </c>
+      <c r="N148" t="n">
+        <v>0</v>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>C-020</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Wach had ttobis kaydouz 3la Jame3 lfna?</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>واش هاد الطوبيس كيدوز على جامع الفنا؟</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr"/>
+      <c r="N149" t="n">
+        <v>0</v>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>C-021</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>الخدمة كاينة ولكن خاص بنادم يصبر ويزير راسو.</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Lkhedma kayna walakin khas bnadem yssber w yzeyyer rassou.</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>lkhdma kayna walakin khass bnadem ysber.|lkhedma kayna walakin khas bnadm ysber.</t>
+        </is>
+      </c>
+      <c r="N150" t="n">
+        <v>0</v>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>C-021</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Lkhedma kayna walakin khas bnadem yssber w yzeyyer rassou.</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>الخدمة كاينة ولكن خاص بنادم يصبر ويزير راسو.</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr"/>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>C-022</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>نقص ليا شوية فالثمن راني كليان قديم عندك.</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>N9es lia chwiya f ttaman rani klyan 9dim 3ndek.</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>n9es liya chwia f taman rani cliyan qdim 3ndk.|n9es lia chwiya f taman.</t>
+        </is>
+      </c>
+      <c r="N152" t="n">
+        <v>0</v>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>achats</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>C-022</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>N9es lia chwiya f ttaman rani klyan 9dim 3ndek.</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>نقص ليا شوية فالثمن راني كليان قديم عندك.</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr"/>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>achats</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>C-023</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>سد الشرجم راه كيدخل البرد بزاف لبيت النعاس.</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Sedd ccherjem rah kaydkhol lberd bzaf l bit nna3s.</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>sedd cherjam rah kaydkhol lberd bzaf.|sed cherjem rah kidkhol lberd.</t>
+        </is>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>maison</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>C-023</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Sedd ccherjem rah kaydkhol lberd bzaf l bit nna3s.</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>سد الشرجم راه كيدخل البرد بزاف لبيت النعاس.</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr"/>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>maison</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>C-024</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>الويفي تقيل بزاف اليوم، واقيلا خاصنا نروديماريو الروتور.</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Lwifi t9il bzaf lyoma, wa9ila khasna nredemariw lrouteur.</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>lwifi tqil bzaf lyom, waqila khassna nredemariw routeur.|l wifi t9il bzaf lyoma.</t>
+        </is>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>technologie</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>C-024</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Lwifi t9il bzaf lyoma, wa9ila khasna nredemariw lrouteur.</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>الويفي تقيل بزاف اليوم، واقيلا خاصنا نروديماريو الروتور.</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr"/>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>technologie</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs & chore: README complet, registre decisions.md, hygiene et scores normalises
</commit_message>
<xml_diff>
--- a/data/final/benchmark.xlsx
+++ b/data/final/benchmark.xlsx
@@ -536,13 +536,13 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>مشا أحمد للحانوت فالصباح، شرا الخبز والحليب. ملي رجع، لقا مو كتسناه باش يفطرو.</t>
+          <t>مشا أحمد للحانوت فالصباح, شرا الخبز والحليب. ملي رجع, لقا مو كتسناه باش يفطرو.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>شنو شرا أحمد؟</t>
+          <t>شنو شرا أحمد?</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -706,13 +706,13 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>فاطمة عيانة بزاف اليوم، فيها السخانة وراها ناعسة فالدار وممشاتش للخدمة.</t>
+          <t>فاطمة عيانة بزاف اليوم, فيها السخانة وراها ناعسة فالدار وممشاتش للخدمة.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>علاش فاطمة ممشاتش للخدمة؟</t>
+          <t>علاش فاطمة ممشاتش للخدمة?</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -876,13 +876,13 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ياسين كيقرا فكلية العلوم، كل نهار كياخد الطرامواي مع السبعة باش مايوصلش معطل.</t>
+          <t>ياسين كيقرا فكلية العلوم, كل نهار كياخد الطرامواي مع السبعة باش مايوصلش معطل.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>باش كيمشي ياسين للكلية؟</t>
+          <t>باش كيمشي ياسين للكلية?</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1046,13 +1046,13 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>الجو زوين هاد الويكاند فالرباط، والناس خرجو كاملين يتساراو فلوضاية ويتبرعو بالهوا د البحر.</t>
+          <t>الجو زوين هاد الويكاند فالرباط, والناس خرجو كاملين يتساراو فلوضاية ويتبرعو بالهوا د البحر.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>فين مشاو الناس يتساراو؟</t>
+          <t>فين مشاو الناس يتساراو?</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1216,13 +1216,13 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>كريم عندو امتحان السيمانة الجاية، طفا التلفزة والتلفون وبدا كيراجع دروسو مزيان.</t>
+          <t>كريم عندو امتحان السيمانة الجاية, طفا التلفزة والتلفون وبدا كيراجع دروسو مزيان.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>شنو دار كريم باش يراجع؟</t>
+          <t>شنو دار كريم باش يراجع?</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1386,13 +1386,13 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>فاطمة فاقت مع السبعة، وجدت راسها ومشات للمدرسة. ملي وصلات، لقات القسم مسدود حيث الأستاذ مريض.</t>
+          <t>فاطمة فاقت مع السبعة, وجدت راسها ومشات للمدرسة. ملي وصلات, لقات القسم مسدود حيث الأستاذ مريض.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>علاش ما قراوش التلاميذ؟</t>
+          <t>علاش ما قراوش التلاميذ?</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1556,13 +1556,13 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>الباب د الدار تبلوكا وما بغاش يتحل، عيطنا على النجار جا فالصباح صاوب الساقطة.</t>
+          <t>الباب د الدار تبلوكا وما بغاش يتحل, عيطنا على النجار جا فالصباح صاوب الساقطة.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>شكون صاوب الباب؟</t>
+          <t>شكون صاوب الباب?</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1726,13 +1726,13 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>مريم كتوجد للحفلة د التخرج ديالها، شرات قفطان غوز وطالون باش تبان زوينة.</t>
+          <t>مريم كتوجد للحفلة د التخرج ديالها, شرات قفطان غوز وطالون باش تبان زوينة.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>شنو شرات مريم للحفلة؟</t>
+          <t>شنو شرات مريم للحفلة?</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1902,7 +1902,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>علاش تعطل القطار؟</t>
+          <t>علاش تعطل القطار?</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2066,13 +2066,13 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ملي دخل البرد، مشات العائلة كلها شربات بصارة سخونة بالزيت البلدية والكامون.</t>
+          <t>ملي دخل البرد, مشات العائلة كلها شربات بصارة سخونة بالزيت البلدية والكامون.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>شنو شربات العائلة؟</t>
+          <t>شنو شربات العائلة?</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>فين غادي تمشي فهاد العطلة؟</t>
+          <t>فين غادي تمشي فهاد العطلة?</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>فين غادي تمشي فهاد العطلة؟</t>
+          <t>فين غادي تمشي فهاد العطلة?</t>
         </is>
       </c>
       <c r="M49" t="inlineStr"/>
@@ -4428,7 +4428,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>سمح ليا، واش كتعرف فين كاين البنك؟</t>
+          <t>سمح ليا, واش كتعرف فين كاين البنك?</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -4508,7 +4508,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>سمح ليا، واش كتعرف فين كاين البنك؟</t>
+          <t>سمح ليا, واش كتعرف فين كاين البنك?</t>
         </is>
       </c>
       <c r="M55" t="inlineStr"/>
@@ -4696,7 +4696,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>شحال كيدير هاد الكيلو ديال التفاح؟</t>
+          <t>شحال كيدير هاد الكيلو ديال التفاح?</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -4776,7 +4776,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>شحال كيدير هاد الكيلو ديال التفاح؟</t>
+          <t>شحال كيدير هاد الكيلو ديال التفاح?</t>
         </is>
       </c>
       <c r="M59" t="inlineStr"/>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>تبارك الله عليك، راك خدمتي مزيان فهاد المشروع.</t>
+          <t>تبارك الله عليك, راك خدمتي مزيان فهاد المشروع.</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -5044,7 +5044,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>تبارك الله عليك، راك خدمتي مزيان فهاد المشروع.</t>
+          <t>تبارك الله عليك, راك خدمتي مزيان فهاد المشروع.</t>
         </is>
       </c>
       <c r="M63" t="inlineStr"/>
@@ -5232,13 +5232,13 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>حميد ضرّاتو ضرسة العقل، مشا عند دونتيست فالعشية حيدها ليه وعطاه الدوا.</t>
+          <t>حميد ضرّاتو ضرسة العقل, مشا عند دونتيست فالعشية حيدها ليه وعطاه الدوا.</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>شنو دار حميد عند الطبيب؟</t>
+          <t>شنو دار حميد عند الطبيب?</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -5402,13 +5402,13 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>رشيد مشا للمقاطعة باش يصادق على العقد، لقا الزحام بزاف وتسنى نوبتو حتى لتماش.</t>
+          <t>رشيد مشا للمقاطعة باش يصادق على العقد, لقا الزحام بزاف وتسنى نوبتو حتى لتماش.</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>علاش مشا رشيد للمقاطعة؟</t>
+          <t>علاش مشا رشيد للمقاطعة?</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -5572,13 +5572,13 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>المنتخب المغربي ربح الماتش بجوج لواحد، وسجل النصيري هدف واعر بالراس فالشوط الثاني.</t>
+          <t>المنتخب المغربي ربح الماتش بجوج لواحد, وسجل النصيري هدف واعر بالراس فالشوط الثاني.</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>كيفاش تسجل الهدف ديال النصيري؟</t>
+          <t>كيفاش تسجل الهدف ديال النصيري?</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -5742,13 +5742,13 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>نهار الجمعة، جمعات الوالدة العائلة كلها ودارت ليهم قصعة د كسكسو بالسبع خضاري واللبن.</t>
+          <t>نهار الجمعة, جمعات الوالدة العائلة كلها ودارت ليهم قصعة د كسكسو بالسبع خضاري واللبن.</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>شنو وجدات الوالدة نهار الجمعة؟</t>
+          <t>شنو وجدات الوالدة نهار الجمعة?</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -5912,13 +5912,13 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>طاحت الشتا خيط من السما، الشوارع فايضين والناس هازين المظلات كيجريو للديور.</t>
+          <t>طاحت الشتا خيط من السما, الشوارع فايضين والناس هازين المظلات كيجريو للديور.</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>كيفاش كان الحال على برا؟</t>
+          <t>كيفاش كان الحال على برا?</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6082,13 +6082,13 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>التلفون ديال أنس طاح ليه فالما وتطفى، داه للمصلح بدّل ليه لافيشور ورجع خدام.</t>
+          <t>التلفون ديال أنس طاح ليه فالما وتطفى, داه للمصلح بدّل ليه لافيشور ورجع خدام.</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>شنو بدّل المصلح فالتلفون؟</t>
+          <t>شنو بدّل المصلح فالتلفون?</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>فين وصلتي، راني كنتسناك حدا المحطة.</t>
+          <t>فين وصلتي, راني كنتسناك حدا المحطة.</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -7160,7 +7160,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>فين وصلتي، راني كنتسناك حدا المحطة.</t>
+          <t>فين وصلتي, راني كنتسناك حدا المحطة.</t>
         </is>
       </c>
       <c r="M91" t="inlineStr"/>
@@ -7482,7 +7482,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>عفاك شحال الحساب كامل؟</t>
+          <t>عفاك شحال الحساب كامل?</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -7562,7 +7562,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>عفاك شحال الحساب كامل؟</t>
+          <t>عفاك شحال الحساب كامل?</t>
         </is>
       </c>
       <c r="M97" t="inlineStr"/>
@@ -7616,13 +7616,13 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>طارق مشا لكيشي أوطوماتيك باش يخرج الفلوس، لقا الكارت تبلوكات حيت غلط فالمودباس تلاتة د المرات.</t>
+          <t>طارق مشا لكيشي أوطوماتيك باش يخرج الفلوس, لقا الكارت تبلوكات حيت غلط فالمودباس تلاتة د المرات.</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>علاش تبلوكات لاكارت د طارق؟</t>
+          <t>علاش تبلوكات لاكارت د طارق?</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -7786,13 +7786,13 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>سعاد شرات زربية تقليدية د تازناخت من المدينة القديمة ف فاس، صاوبوها بالصوف الحر والألوان الطبيعية.</t>
+          <t>سعاد شرات زربية تقليدية د تازناخت من المدينة القديمة ف فاس, صاوبوها بالصوف الحر والألوان الطبيعية.</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>باش تصاوبات الزربية لي شرات سعاد؟</t>
+          <t>باش تصاوبات الزربية لي شرات سعاد?</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -7956,13 +7956,13 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>الطلبة كراو برطمة قريبة للفاك ب تلتالاف درهم للشهر، مقسومة عليهم بربعة ومفرشة كاملة.</t>
+          <t>الطلبة كراو برطمة قريبة للفاك ب تلتالاف درهم للشهر, مقسومة عليهم بربعة ومفرشة كاملة.</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>بشحال كراو الطلبة البرطمة؟</t>
+          <t>بشحال كراو الطلبة البرطمة?</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -8126,13 +8126,13 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>ملي كان هشام صايغ فلوطوروت، تفشات ليه الرويضة الورانية، وقف فالبان ديرجونس وبدلها بالسوكوندير.</t>
+          <t>ملي كان هشام صايغ فلوطوروت, تفشات ليه الرويضة الورانية, وقف فالبان ديرجونس وبدلها بالسوكوندير.</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>شنو وقع لطوموبيل د هشام؟</t>
+          <t>شنو وقع لطوموبيل د هشام?</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>واش عندك الصرف ديال ميتين درهم؟</t>
+          <t>واش عندك الصرف ديال ميتين درهم?</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -9606,7 +9606,7 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>واش عندك الصرف ديال ميتين درهم؟</t>
+          <t>واش عندك الصرف ديال ميتين درهم?</t>
         </is>
       </c>
       <c r="M125" t="inlineStr"/>
@@ -9660,13 +9660,13 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>سلوى مشات لسنتر فيل تشري كادو لعيد ميلاد ختها، لقات صاك جلد كحل واعر وشراتو.</t>
+          <t>سلوى مشات لسنتر فيل تشري كادو لعيد ميلاد ختها, لقات صاك جلد كحل واعر وشراتو.</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>شنو شرات سلوى كادو لختها؟</t>
+          <t>شنو شرات سلوى كادو لختها?</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -9695,8 +9695,10 @@
         </is>
       </c>
       <c r="M126" t="inlineStr"/>
-      <c r="N126" t="n">
-        <v>0</v>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O126" t="inlineStr">
         <is>
@@ -9778,8 +9780,10 @@
         </is>
       </c>
       <c r="M127" t="inlineStr"/>
-      <c r="N127" t="n">
-        <v>0</v>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O127" t="inlineStr">
         <is>
@@ -9826,13 +9830,13 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>الطاكسي كبير وقف فالرونبوان باش يركب الناس، وبقات بلاصة وحدة اللور خاوية.</t>
+          <t>الطاكسي كبير وقف فالرونبوان باش يركب الناس, وبقات بلاصة وحدة اللور خاوية.</t>
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>فين بقات البلاصة الخاوية فالطاكسي؟</t>
+          <t>فين بقات البلاصة الخاوية فالطاكسي?</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -9861,8 +9865,10 @@
         </is>
       </c>
       <c r="M128" t="inlineStr"/>
-      <c r="N128" t="n">
-        <v>0</v>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O128" t="inlineStr">
         <is>
@@ -9944,8 +9950,10 @@
         </is>
       </c>
       <c r="M129" t="inlineStr"/>
-      <c r="N129" t="n">
-        <v>0</v>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -9992,13 +10000,13 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>مشاو الدراري للبحر فالصيف، لقاوه عامر والموج عالي بزاف حيت كان الريح الشرقي.</t>
+          <t>مشاو الدراري للبحر فالصيف, لقاوه عامر والموج عالي بزاف حيت كان الريح الشرقي.</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>علاش كان الموج عالي فالبحر؟</t>
+          <t>علاش كان الموج عالي فالبحر?</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -10027,8 +10035,10 @@
         </is>
       </c>
       <c r="M130" t="inlineStr"/>
-      <c r="N130" t="n">
-        <v>0</v>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -10110,8 +10120,10 @@
         </is>
       </c>
       <c r="M131" t="inlineStr"/>
-      <c r="N131" t="n">
-        <v>0</v>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -10158,13 +10170,13 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>جواد نسى السوارت فوق الطابلة فالكوزينة، وملي خرج وسد الباب عاد تفكرهم وبقا واحل.</t>
+          <t>جواد نسى السوارت فوق الطابلة فالكوزينة, وملي خرج وسد الباب عاد تفكرهم وبقا واحل.</t>
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>فين نسى جواد السوارت؟</t>
+          <t>فين نسى جواد السوارت?</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -10193,8 +10205,10 @@
         </is>
       </c>
       <c r="M132" t="inlineStr"/>
-      <c r="N132" t="n">
-        <v>0</v>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -10276,8 +10290,10 @@
         </is>
       </c>
       <c r="M133" t="inlineStr"/>
-      <c r="N133" t="n">
-        <v>0</v>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -10343,8 +10359,10 @@
         </is>
       </c>
       <c r="M134" t="inlineStr"/>
-      <c r="N134" t="n">
-        <v>0</v>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -10410,8 +10428,10 @@
         </is>
       </c>
       <c r="M135" t="inlineStr"/>
-      <c r="N135" t="n">
-        <v>0</v>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O135" t="inlineStr">
         <is>
@@ -10477,8 +10497,10 @@
         </is>
       </c>
       <c r="M136" t="inlineStr"/>
-      <c r="N136" t="n">
-        <v>0</v>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O136" t="inlineStr">
         <is>
@@ -10544,8 +10566,10 @@
         </is>
       </c>
       <c r="M137" t="inlineStr"/>
-      <c r="N137" t="n">
-        <v>0</v>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -10611,8 +10635,10 @@
         </is>
       </c>
       <c r="M138" t="inlineStr"/>
-      <c r="N138" t="n">
-        <v>0</v>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -10678,8 +10704,10 @@
         </is>
       </c>
       <c r="M139" t="inlineStr"/>
-      <c r="N139" t="n">
-        <v>0</v>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -10745,8 +10773,10 @@
         </is>
       </c>
       <c r="M140" t="inlineStr"/>
-      <c r="N140" t="n">
-        <v>0</v>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O140" t="inlineStr">
         <is>
@@ -10812,8 +10842,10 @@
         </is>
       </c>
       <c r="M141" t="inlineStr"/>
-      <c r="N141" t="n">
-        <v>0</v>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -10879,8 +10911,10 @@
         </is>
       </c>
       <c r="M142" t="inlineStr"/>
-      <c r="N142" t="n">
-        <v>0</v>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -10946,8 +10980,10 @@
         </is>
       </c>
       <c r="M143" t="inlineStr"/>
-      <c r="N143" t="n">
-        <v>0</v>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O143" t="inlineStr">
         <is>
@@ -11013,8 +11049,10 @@
         </is>
       </c>
       <c r="M144" t="inlineStr"/>
-      <c r="N144" t="n">
-        <v>0</v>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O144" t="inlineStr">
         <is>
@@ -11080,8 +11118,10 @@
         </is>
       </c>
       <c r="M145" t="inlineStr"/>
-      <c r="N145" t="n">
-        <v>0</v>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O145" t="inlineStr">
         <is>
@@ -11128,7 +11168,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>ما بقاش فيا الحال، المهم هي الصحة والسلامة.</t>
+          <t>ما بقاش فيا الحال, المهم هي الصحة والسلامة.</t>
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
@@ -11147,8 +11187,10 @@
           <t>mab9ach fia lhal, lmohim hya seha w salama.|ma b9ach fiya lhal.</t>
         </is>
       </c>
-      <c r="N146" t="n">
-        <v>0</v>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O146" t="inlineStr">
         <is>
@@ -11206,12 +11248,14 @@
       <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr">
         <is>
-          <t>ما بقاش فيا الحال، المهم هي الصحة والسلامة.</t>
+          <t>ما بقاش فيا الحال, المهم هي الصحة والسلامة.</t>
         </is>
       </c>
       <c r="M147" t="inlineStr"/>
-      <c r="N147" t="n">
-        <v>0</v>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -11258,7 +11302,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>واش هاد الطوبيس كيدوز على جامع الفنا؟</t>
+          <t>واش هاد الطوبيس كيدوز على جامع الفنا?</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -11277,8 +11321,10 @@
           <t>wach had tobis kidouz 3la jama3 lfna?|wach had ttobis kaydoz 3la jame3 lfna?</t>
         </is>
       </c>
-      <c r="N148" t="n">
-        <v>0</v>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -11336,12 +11382,14 @@
       <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr">
         <is>
-          <t>واش هاد الطوبيس كيدوز على جامع الفنا؟</t>
+          <t>واش هاد الطوبيس كيدوز على جامع الفنا?</t>
         </is>
       </c>
       <c r="M149" t="inlineStr"/>
-      <c r="N149" t="n">
-        <v>0</v>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O149" t="inlineStr">
         <is>
@@ -11407,8 +11455,10 @@
           <t>lkhdma kayna walakin khass bnadem ysber.|lkhedma kayna walakin khas bnadm ysber.</t>
         </is>
       </c>
-      <c r="N150" t="n">
-        <v>0</v>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O150" t="inlineStr">
         <is>
@@ -11470,8 +11520,10 @@
         </is>
       </c>
       <c r="M151" t="inlineStr"/>
-      <c r="N151" t="n">
-        <v>0</v>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -11537,8 +11589,10 @@
           <t>n9es liya chwia f taman rani cliyan qdim 3ndk.|n9es lia chwiya f taman.</t>
         </is>
       </c>
-      <c r="N152" t="n">
-        <v>0</v>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O152" t="inlineStr">
         <is>
@@ -11600,8 +11654,10 @@
         </is>
       </c>
       <c r="M153" t="inlineStr"/>
-      <c r="N153" t="n">
-        <v>0</v>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -11667,8 +11723,10 @@
           <t>sedd cherjam rah kaydkhol lberd bzaf.|sed cherjem rah kidkhol lberd.</t>
         </is>
       </c>
-      <c r="N154" t="n">
-        <v>0</v>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -11730,8 +11788,10 @@
         </is>
       </c>
       <c r="M155" t="inlineStr"/>
-      <c r="N155" t="n">
-        <v>0</v>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O155" t="inlineStr">
         <is>
@@ -11778,7 +11838,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>الويفي تقيل بزاف اليوم، واقيلا خاصنا نروديماريو الروتور.</t>
+          <t>الويفي تقيل بزاف اليوم, واقيلا خاصنا نروديماريو الروتور.</t>
         </is>
       </c>
       <c r="F156" t="inlineStr"/>
@@ -11797,8 +11857,10 @@
           <t>lwifi tqil bzaf lyom, waqila khassna nredemariw routeur.|l wifi t9il bzaf lyoma.</t>
         </is>
       </c>
-      <c r="N156" t="n">
-        <v>0</v>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -11856,12 +11918,14 @@
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr">
         <is>
-          <t>الويفي تقيل بزاف اليوم، واقيلا خاصنا نروديماريو الروتور.</t>
+          <t>الويفي تقيل بزاف اليوم, واقيلا خاصنا نروديماريو الروتور.</t>
         </is>
       </c>
       <c r="M157" t="inlineStr"/>
-      <c r="N157" t="n">
-        <v>0</v>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="O157" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs & ui: finalisation du poster ICAIS'26, README et finitions dashboard
</commit_message>
<xml_diff>
--- a/data/final/benchmark.xlsx
+++ b/data/final/benchmark.xlsx
@@ -3975,7 +3975,11 @@
           <t>عجبني هاد الفيلم بزاف.</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>عجبني هذا الفيلم بزاف|عجبني هاد الفلم بزاف</t>
+        </is>
+      </c>
       <c r="N47" t="inlineStr">
         <is>
           <t>0</t>
@@ -4109,7 +4113,11 @@
           <t>فين غادي تمشي فهاد العطلة?</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>فين غادي تمشي فهاد العطله?|فين غتمشي فهاد العطلة?</t>
+        </is>
+      </c>
       <c r="N49" t="inlineStr">
         <is>
           <t>0</t>
@@ -4243,7 +4251,11 @@
           <t>الماكلة ديال هاد الريسطو بنينة ونقية.</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>الماكله ديال هاد الريسطو بنينه ونقيه|الماكلة د هاد الريسطو بنينة ونقية</t>
+        </is>
+      </c>
       <c r="N51" t="inlineStr">
         <is>
           <t>0</t>
@@ -4377,7 +4389,11 @@
           <t>ما كرهتش نشرب كاس د أتاي مشحر.</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ما كرهتش نشرب كاس ديال اتاي مشحر|ماكرهتش نشرب كاس د اتاي مشحر</t>
+        </is>
+      </c>
       <c r="N53" t="inlineStr">
         <is>
           <t>0</t>
@@ -4511,7 +4527,11 @@
           <t>سمح ليا, واش كتعرف فين كاين البنك?</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>سمح لي, واش كتعرف فين كاين البنك?|سمحي ليا واش كتعرف فين كاين البنك?</t>
+        </is>
+      </c>
       <c r="N55" t="inlineStr">
         <is>
           <t>0</t>
@@ -4645,7 +4665,11 @@
           <t>بغيت نمشي للسوق بكري.</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>بغيت نمشي للسوق بكري|بغيت نمشي لسوق بكري</t>
+        </is>
+      </c>
       <c r="N57" t="inlineStr">
         <is>
           <t>0</t>
@@ -4779,7 +4803,11 @@
           <t>شحال كيدير هاد الكيلو ديال التفاح?</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>شحال كيدير هذا الكيلو ديال التفاح?|شحال كيدير هاد الكيلو د التفاح?</t>
+        </is>
+      </c>
       <c r="N59" t="inlineStr">
         <is>
           <t>0</t>
@@ -4913,7 +4941,11 @@
           <t>بغيت نسولك على التوقيت ديال الخدمة غدا.</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>بغيت نسولك على التوقيت ديال الخدمه غدا|بغيت نسولك على وقت الخدمة غدا</t>
+        </is>
+      </c>
       <c r="N61" t="inlineStr">
         <is>
           <t>0</t>
@@ -5047,7 +5079,11 @@
           <t>تبارك الله عليك, راك خدمتي مزيان فهاد المشروع.</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>تبارك الله عليك راك خدمتي مزيان فهاد المشروع|تبارك الله عليك خدمتي مزيان فهاد المشروع</t>
+        </is>
+      </c>
       <c r="N63" t="inlineStr">
         <is>
           <t>0</t>
@@ -5181,7 +5217,11 @@
           <t>كنتمنى ليك التوفيق والنجاح فالامتحان ديالك.</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>كنتمنى لك التوفيق والنجاح فالامتحان ديالك|كنتمنى ليك التوفيق والنجاح في الامتحان ديالك</t>
+        </is>
+      </c>
       <c r="N65" t="inlineStr">
         <is>
           <t>0</t>
@@ -7163,7 +7203,11 @@
           <t>فين وصلتي, راني كنتسناك حدا المحطة.</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr"/>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>فين وصلتي راني كنتسناك حدا المحطه|فين وصلتي راني كنتسناك عند المحطة</t>
+        </is>
+      </c>
       <c r="N91" t="inlineStr">
         <is>
           <t>0</t>
@@ -7297,7 +7341,11 @@
           <t>خاصك تشرب الدوا فوقتو وتبع الريجيم.</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr"/>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>خاصك تشرب الدوا في وقته وتبع الريجيم|خاصك تشرب الدواء فوقتو وتبع الريجيم</t>
+        </is>
+      </c>
       <c r="N93" t="inlineStr">
         <is>
           <t>0</t>
@@ -7431,7 +7479,11 @@
           <t>صيفط ليا الإيميل باش نشوف الدوسي اليوم.</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>صيفط ليا الايميل باش نشوف الدوسي اليوم|صيفط لي ليميل باش نشوف الدوسي اليوم</t>
+        </is>
+      </c>
       <c r="N95" t="inlineStr">
         <is>
           <t>0</t>
@@ -7565,7 +7617,11 @@
           <t>عفاك شحال الحساب كامل?</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr"/>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>عفاك شحال الحساب كامل?|عافاك شحال الحساب كامل?</t>
+        </is>
+      </c>
       <c r="N97" t="inlineStr">
         <is>
           <t>0</t>
@@ -9207,7 +9263,11 @@
           <t>الله يعطيك الصحة على هاد المجهود.</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr"/>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>الله يعطيك الصحه على هاد المجهود|الله يعطيك الصحة على هذا المجهود</t>
+        </is>
+      </c>
       <c r="N119" t="inlineStr">
         <is>
           <t>0</t>
@@ -9341,7 +9401,11 @@
           <t>كاين واحد الصهد صعيب اليوم فالزنقة.</t>
         </is>
       </c>
-      <c r="M121" t="inlineStr"/>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>كاين واحد الصهد صعيب اليوم فالزنقه|كاين واحد الصهد صعيب اليوم فالشارع</t>
+        </is>
+      </c>
       <c r="N121" t="inlineStr">
         <is>
           <t>0</t>
@@ -9475,7 +9539,11 @@
           <t>سلم ليا على الوالد والدار كاملين.</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr"/>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>سلم ليا على الوالد والعائله كاملين|سلم ليا على الواليد والدار كاملين</t>
+        </is>
+      </c>
       <c r="N123" t="inlineStr">
         <is>
           <t>0</t>
@@ -9609,7 +9677,11 @@
           <t>واش عندك الصرف ديال ميتين درهم?</t>
         </is>
       </c>
-      <c r="M125" t="inlineStr"/>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>واش عندك الصرف ديال مائتين درهم?|واش عندك الصرف د ميتين درهم?</t>
+        </is>
+      </c>
       <c r="N125" t="inlineStr">
         <is>
           <t>0</t>
@@ -11251,7 +11323,11 @@
           <t>ما بقاش فيا الحال, المهم هي الصحة والسلامة.</t>
         </is>
       </c>
-      <c r="M147" t="inlineStr"/>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>ما بقاش فيا الحال المهم هي الصحه والسلامه|مابقاش فيا الحال المهم هي الصحة والسلامة</t>
+        </is>
+      </c>
       <c r="N147" t="inlineStr">
         <is>
           <t>0</t>
@@ -11385,7 +11461,11 @@
           <t>واش هاد الطوبيس كيدوز على جامع الفنا?</t>
         </is>
       </c>
-      <c r="M149" t="inlineStr"/>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>واش هاد الطوبيس كيدوز على جامع الفنا?|واش هذا الطوبيس كيدوز على جامع الفنا?</t>
+        </is>
+      </c>
       <c r="N149" t="inlineStr">
         <is>
           <t>0</t>
@@ -11519,7 +11599,11 @@
           <t>الخدمة كاينة ولكن خاص بنادم يصبر ويزير راسو.</t>
         </is>
       </c>
-      <c r="M151" t="inlineStr"/>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>الخدمه كاينة ولكن خاص بنادم يصبر ويزير راسو|الخدمة كاينة ولكن خاص الواحد يصبر</t>
+        </is>
+      </c>
       <c r="N151" t="inlineStr">
         <is>
           <t>0</t>
@@ -11653,7 +11737,11 @@
           <t>نقص ليا شوية فالثمن راني كليان قديم عندك.</t>
         </is>
       </c>
-      <c r="M153" t="inlineStr"/>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>نقص ليا شويه فالثمن راني كليان قديم عندك|نقص لي شوية فالثمن راني كليان قديم</t>
+        </is>
+      </c>
       <c r="N153" t="inlineStr">
         <is>
           <t>0</t>
@@ -11787,7 +11875,11 @@
           <t>سد الشرجم راه كيدخل البرد بزاف لبيت النعاس.</t>
         </is>
       </c>
-      <c r="M155" t="inlineStr"/>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>سد الشرجم راه كيدخل البرد بزاف لبيت النعاس|سد الشرجم راه كيدخل البرد لبيت النعاس</t>
+        </is>
+      </c>
       <c r="N155" t="inlineStr">
         <is>
           <t>0</t>
@@ -11921,7 +12013,11 @@
           <t>الويفي تقيل بزاف اليوم, واقيلا خاصنا نروديماريو الروتور.</t>
         </is>
       </c>
-      <c r="M157" t="inlineStr"/>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>الويفي ثقيل بزاف اليوم واقيلا خاصنا نروديماريو الروتور|الويفي تقيل بزاف اليوم خاصنا نروديماريو الروتور</t>
+        </is>
+      </c>
       <c r="N157" t="inlineStr">
         <is>
           <t>0</t>

</xml_diff>

<commit_message>
feat(figures): mise a jour officielle figure N=27 paires et McNemar p=0.0215
</commit_message>
<xml_diff>
--- a/data/final/benchmark.xlsx
+++ b/data/final/benchmark.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S157"/>
+  <dimension ref="A1:S191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12045,6 +12045,2476 @@
       </c>
       <c r="S157" t="inlineStr"/>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Q-025</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>سعيد شرا تلفازة ذكية، ولكن ملي وصل لدار لقا التيليكوموند ناقصة فالكرطونة، فرجع للحانوت يبدلها.</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>علاش رجع سعيد للحانوت فالبلاصة؟</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>حيت التلفازة لقاها مهرسة</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>حيت الصورة ما واضحاش بزاف</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>حيت ناقصة التيليكوموند تما</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>حيت بغا يرجع كاع فلوسو دابا</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr"/>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>commerce</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Q-025</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Sa3id chra talvaza dkiya, walakin mlli wsel lddar l9a ttélécommande na9sa f lkartouna, rje3 l l7anout ybeddelha.</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>3lach rje3 Sa3id l l7anout flblassa?</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>7it ttalvaza l9aha mherrsa</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>7it ssoura ma wadhach bzaf</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>7it na9sa ttélécommande tmma</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>7it bgha yrje3 ga3 flouso daba</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr"/>
+      <c r="N159" t="n">
+        <v>0</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>commerce</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Q-026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>المدير طلب من الموظفين يحبسو الخدمة بكري حيت كاين انقطاع ديال الضو مبرمج فالزنقة مع الجوج.</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>شنو هو السبب لتوقيف الخدمة؟</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>حيت الضو غادي يتقطع تماك</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>حيت كاين اجتماع طارئ دابا</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>حيت سالات ساعات الخدمة رسميا</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>حيت الموظفين جاو عيانين اليوم</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr"/>
+      <c r="N160" t="n">
+        <v>0</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Q-026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Lmodir tleb mn lmowaddafin y7ebso lkhedma bekri 7it kayn in9ita3 dyal ddow mbermej f zzen9a m3a jjoj.</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Chnou houwa ssabab l tw9if lkhedma?</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>7it ddow ghadi yt9te3 tmmak</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>7it kayn ijtima3 tari2 daba</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>7it salat sa3at lkhedma rsemiyan</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>7it lmowaddafin jaw 3yanin lyoma</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr"/>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Q-027</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>يونس كان غادي للمطار، ولكن لقا لوطوروت مبلوكية بحادثة سير، فاضطر يدوز من الطريق الوطنية.</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>علاش بدل يونس الطريق ديالو؟</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>حيت سالا ليه المازوط فالطريق</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>حيت الطوموبيل سخنات ليه بزاف</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>حيت بغا يشوف صاحبو فالطريق</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>حيت لوطوروت تبلوكات بحادثة</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr"/>
+      <c r="N162" t="n">
+        <v>0</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Q-027</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Younes kan ghadi l lmatar, walakin l9a l'autoroute mbloukiya b 7adita d ssir, f dtar ydouz mn tri9 lwataniya.</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>3lach beddel Younes tri9 dyalo?</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>7it sala lih lmazot f tri9</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>7it ttomobil skhnat lih bzaf</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>7it bgha ychouf sa7bo f tri9</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>7it l'autoroute tbloukat b 7adita</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr"/>
+      <c r="N163" t="n">
+        <v>0</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Q-028</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>الطبيب نصح مصطفى يحبس السكر والملحة وينقص من الخبز الأبيض باش يهبط ليه الطانسيو.</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>شنو خاص يدير مصطفى باش يبرى؟</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>خاصو يشرب القهوة بزاف ديما</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>خاصو ينقص السكر والملحة والخبز</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>خاصو ينعس النهار كامل فالدار</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>خاصو يسافر للبحر يبدل الجو</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr"/>
+      <c r="N164" t="n">
+        <v>0</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Q-028</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Ttbib nse7 Mostafa y7bes ssokkar w lmel7a w yn9es mn lkhobz lbyed bach yhbet lih ttansyou.</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Chnou khas ydir Mostafa bach ybra?</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>khaso ychreb l9ahwa bzaf dima</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>khaso yn9es ssokkar w lmel7a w lkhobz</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>khaso yn3es nnhar kamel f ddar</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>khaso ysafer l lb7ar ybeddel ljow</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr"/>
+      <c r="N165" t="n">
+        <v>0</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Q-029</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>الأستاذ لغى الحصة ديال الماط العشية حيت عندو اجتماع عاجل مع الإدارة د الكلية.</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>علاش تلغات الحصة د الماط؟</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>حيت القاعة لقاها عامرة بناس</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>حيت الطلبة غابو كاملين اليوم</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>حيت عندو اجتماع مع الإدارة</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>حيت ترونات السيمانة د العطلة</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr"/>
+      <c r="N166" t="n">
+        <v>0</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Q-029</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>L'prof lgha l7essa dyal lmath l3chiya 7it 3ndo ijtima3 3ajil m3a l'idara d lkollia.</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>3lach tlghat l7essa d lmath?</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>7it l9a3a l9aha 3amra b nass</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>7it ttolaba ghabo kamlin lyoma</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>7it 3ndo ijtima3 m3a l'idara</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>7it trwnat ssimana d l3otla</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr"/>
+      <c r="N167" t="n">
+        <v>0</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>école</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Q-030</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>العائلة كاملة قررات تعيد ف العروبية عند الجد حيت توحشو اللمة د الحباب والأجواء التقليدية.</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>فين قررات العائلة تدوز العيد؟</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>ف العروبية عند الجد الكبير</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>ف لوطيل على البحر فالمدينة</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>ف دارهم فالمدينة بلا سفر</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>ف دار عمهم الصغير فالرباط</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr"/>
+      <c r="N168" t="n">
+        <v>0</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>famille</t>
+        </is>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Q-030</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>qcm</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>L3a2ila kamla 9errrat t3eyyed f l3roubiya 3nd jjdd 7it twa7cho lmma d l7bab w l'ajwa2 tta9lidiya.</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Fin 9errrat l3a2ila ddozewez l3id?</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>f l3roubiya 3nd jjdd lkbir</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>f l'hôtel 3la lb7ar f lmdina</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>f darhom f lmdina bla safer</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>f dar 3mmhom ssghir f Rbat</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr"/>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>famille</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>N-013a</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>حكيم ركب فالتران د الرباط مع العشرة د الصباح.</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>حكيم مسافر على برا د مدينتو.</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr"/>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>N-013a</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Hakim rkeb f ttran d Rbat m3a l3chra d sba7.</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Hakim msafer 3la berra d mdinto.</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr"/>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>N-013b</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>حكيم ركب فالتران د الرباط مع العشرة د الصباح.</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>حكيم جالس دابا فدارو كيتفرج.</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr"/>
+      <c r="N172" t="n">
+        <v>0</v>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>N-013b</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Hakim rkeb f ttran d Rbat m3a l3chra d sba7.</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Hakim jales daba f daro kaytferrej.</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="n">
+        <v>0</v>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>N-013c</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>حكيم ركب فالتران د الرباط مع العشرة د الصباح.</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>حكيم غادي يحضر لعرس ف الرباط.</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr"/>
+      <c r="N174" t="n">
+        <v>0</v>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>N-013c</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Hakim rkeb f ttran d Rbat m3a l3chra d sba7.</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Hakim ghadi ye7der l 3ers f Rbat.</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr"/>
+      <c r="N175" t="n">
+        <v>0</v>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>N-014a</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>نادية شرات الدجاج والحامض مصير والزيتون باش تطيب العشا.</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>نادية كتعرف شنو باغا توجد للعشا.</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr"/>
+      <c r="N176" t="n">
+        <v>0</v>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>N-014a</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Nadia chrat ddjaj w l7amed mssiyer w zzitoun bach ttyeb l3cha.</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Nadia kat3ref chnou bagha twjed l l3cha.</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="n">
+        <v>0</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>N-014b</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>نادية شرات الدجاج والحامض مصير والزيتون باش تطيب العشا.</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>نادية معولة تاكل ف الريسطو الليلة.</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="n">
+        <v>0</v>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>N-014b</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Nadia chrat ddjaj w l7amed mssiyer w zzitoun bach ttyeb l3cha.</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Nadia m3ewla takol f rresto llila.</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="n">
+        <v>0</v>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>N-014c</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>نادية شرات الدجاج والحامض مصير والزيتون باش تطيب العشا.</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>نادية عارضة على دار عمها كاملين.</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="n">
+        <v>0</v>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>N-014c</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Nadia chrat ddjaj w l7amed mssiyer w zzitoun bach ttyeb l3cha.</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Nadia 3arda 3la dar 3mmha kamlin.</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="n">
+        <v>0</v>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>cuisine</t>
+        </is>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>N-015a</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>رضى تقبل ف المنحة الدراسية ف فرنسا وغادي يمشي فالشتنبر.</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>رضى عندو فرصة يقرا على برا.</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr"/>
+      <c r="N182" t="n">
+        <v>0</v>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>N-015a</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Reda t9bel f lmin7a ddirasiya f Fransa w ghadi ymchi f septembre.</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Reda 3ndo forsa y9ra 3la berra.</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr"/>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>implication</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr"/>
+      <c r="N183" t="n">
+        <v>0</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>N-015b</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>رضى تقبل ف المنحة الدراسية ف فرنسا وغادي يمشي فالشتنبر.</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>الدوسي د المنحة د رضى ترفض نهائيا.</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="n">
+        <v>0</v>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>N-015b</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Reda t9bel f lmin7a ddirasiya f Fransa w ghadi ymchi f septembre.</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Ddossier d lmin7a d Reda trefd nihaiyan.</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>contradiction</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="n">
+        <v>0</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>N-015c</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>رضى تقبل ف المنحة الدراسية ف فرنسا وغادي يمشي فالشتنبر.</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>رضى لقا ديجا السكن الجامعي ف باريس.</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr"/>
+      <c r="N186" t="n">
+        <v>0</v>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>N-015c</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>nli</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Reda t9bel f lmin7a ddirasiya f Fransa w ghadi ymchi f septembre.</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Reda l9a déja ssakan ljami3i f Paris.</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr"/>
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>neutre</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr"/>
+      <c r="N187" t="n">
+        <v>0</v>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>éducation</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>C-025</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>راسي كيضرني بزاف خاصني نشرب شي كينة.</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Rassi kayderni bzaf khasni nchreb chi kina.</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>rasi kiderni bzzaf khassni nchrob kina|rassi kaydrni bzaf khasni kina</t>
+        </is>
+      </c>
+      <c r="N188" t="n">
+        <v>0</v>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>C-025</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Rassi kayderni bzaf khasni nchreb chi kina.</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>راسي كيضرني بزاف خاصني نشرب شي كينة.</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>راسي كيضرني بزاف خاصني نشرب كينة|راسي كيضرني بزاف خاصني كينة</t>
+        </is>
+      </c>
+      <c r="N189" t="n">
+        <v>0</v>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>santé</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>C-026</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>ar</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>غدا عندي مقابلة ديال الخدمة مع التسعود الصباح.</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr"/>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Ghedda 3ndi mo9abala dyal lkhedma m3a ttss3oud d sba7.</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>ghda 3ndi entretient d lkhedma m3a 9 sba7|ghedda 3ndi moqabala dial lkhdma</t>
+        </is>
+      </c>
+      <c r="N190" t="n">
+        <v>0</v>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>C-026</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>conversion</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Ghedda 3ndi mo9abala dyal lkhedma m3a ttss3oud d sba7.</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr"/>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>غدا عندي مقابلة ديال الخدمة مع التسعود الصباح.</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>غدا عندي مقابلة د الخدمة مع التسعود د الصباح|غدا عندي مقابلة ديال الخدمة مع 9 د الصباح</t>
+        </is>
+      </c>
+      <c r="N191" t="n">
+        <v>0</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>augmented_native</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>travail</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="S191" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>